<commit_message>
collegamento excel quasi completo
manca contratti, aggiunta contratto e modifica direttamente su excel ecc, manca logo end more user-friendly
</commit_message>
<xml_diff>
--- a/Database_SpiaggiaFacile_Aggiornato.xlsx
+++ b/Database_SpiaggiaFacile_Aggiornato.xlsx
@@ -1,22 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nocer\Documents\UNIVERSITA\1 Triennale UniBG\3 ANNO\9 PROGRAMMAZIONE WEB\PROGETTI\PRIMO\ProgettoWeb-main\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E27A5F3-579C-46FB-B4DC-09FD6DC49F20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10660" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Ombrellone" sheetId="1" r:id="rId1"/>
-    <sheet name="Tipologia" sheetId="2" r:id="rId2"/>
-    <sheet name="Tariffa" sheetId="3" r:id="rId3"/>
-    <sheet name="Cliente" sheetId="4" r:id="rId4"/>
-    <sheet name="Contratto" sheetId="5" r:id="rId5"/>
+    <sheet name="Ombrelloni" sheetId="1" r:id="rId1"/>
+    <sheet name="Tipologie" sheetId="2" r:id="rId2"/>
+    <sheet name="Contratti" sheetId="5" r:id="rId3"/>
+    <sheet name="Tariffa" sheetId="3" r:id="rId4"/>
+    <sheet name="Cliente" sheetId="4" r:id="rId5"/>
     <sheet name="GiornoDisponibilita" sheetId="6" r:id="rId6"/>
     <sheet name="OmbrelloneVenduto" sheetId="7" r:id="rId7"/>
     <sheet name="TipologiaTariffa" sheetId="8" r:id="rId8"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -29,12 +35,6 @@
     <t>settore</t>
   </si>
   <si>
-    <t>numFila</t>
-  </si>
-  <si>
-    <t>numPostoFila</t>
-  </si>
-  <si>
     <t>tipologia</t>
   </si>
   <si>
@@ -194,18 +194,12 @@
     <t>Via Napoli 8</t>
   </si>
   <si>
-    <t>numProgr</t>
-  </si>
-  <si>
     <t>data</t>
   </si>
   <si>
     <t>importo</t>
   </si>
   <si>
-    <t>stipulatoDa</t>
-  </si>
-  <si>
     <t>2025-06-05</t>
   </si>
   <si>
@@ -228,13 +222,25 @@
   </si>
   <si>
     <t>tipoTariffa</t>
+  </si>
+  <si>
+    <t>numero</t>
+  </si>
+  <si>
+    <t>giorni</t>
+  </si>
+  <si>
+    <t>fila</t>
+  </si>
+  <si>
+    <t>PostoFila</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -293,17 +299,25 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -341,7 +355,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -375,6 +389,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -409,9 +424,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -584,11 +600,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -596,21 +612,21 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -619,15 +635,15 @@
         <v>5</v>
       </c>
       <c r="E2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C3">
         <v>2</v>
@@ -636,15 +652,15 @@
         <v>10</v>
       </c>
       <c r="E3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C4">
         <v>3</v>
@@ -653,7 +669,7 @@
         <v>15</v>
       </c>
       <c r="E4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -662,52 +678,52 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
+      <c r="C3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>11</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B4" t="s">
         <v>17</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C4" t="s">
         <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" t="s">
-        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -716,82 +732,64 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>14</v>
+        <v>65</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>23</v>
+        <v>55</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>24</v>
+        <v>56</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B2">
-        <v>20</v>
-      </c>
-      <c r="C2" t="s">
-        <v>31</v>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1001</v>
+      </c>
+      <c r="B2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2">
+        <v>100</v>
       </c>
       <c r="D2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>1002</v>
+      </c>
+      <c r="B3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3">
+        <v>150</v>
+      </c>
+      <c r="D3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>1003</v>
+      </c>
+      <c r="B4" t="s">
         <v>30</v>
       </c>
-      <c r="C3" t="s">
-        <v>32</v>
-      </c>
-      <c r="D3" t="s">
-        <v>35</v>
-      </c>
-      <c r="E3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B4">
-        <v>40</v>
-      </c>
-      <c r="C4" t="s">
-        <v>33</v>
+      <c r="C4">
+        <v>120</v>
       </c>
       <c r="D4" t="s">
-        <v>36</v>
-      </c>
-      <c r="E4" t="s">
-        <v>38</v>
-      </c>
-      <c r="F4">
-        <v>7</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -800,76 +798,82 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2">
+        <v>20</v>
+      </c>
+      <c r="C2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3">
+        <v>30</v>
+      </c>
+      <c r="C3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4">
         <v>40</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" t="s">
-        <v>42</v>
-      </c>
-      <c r="B2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C2" t="s">
-        <v>48</v>
-      </c>
-      <c r="D2" t="s">
-        <v>51</v>
-      </c>
-      <c r="E2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C3" t="s">
-        <v>49</v>
-      </c>
-      <c r="D3" t="s">
-        <v>52</v>
-      </c>
-      <c r="E3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" t="s">
-        <v>44</v>
-      </c>
-      <c r="B4" t="s">
-        <v>47</v>
-      </c>
       <c r="C4" t="s">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="D4" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="E4" t="s">
-        <v>56</v>
+        <v>36</v>
+      </c>
+      <c r="F4">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -878,64 +882,76 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>57</v>
+        <v>12</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>58</v>
+        <v>13</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>59</v>
+        <v>37</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2">
-        <v>1001</v>
+        <v>38</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>40</v>
       </c>
       <c r="B2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C2">
-        <v>100</v>
+        <v>43</v>
+      </c>
+      <c r="C2" t="s">
+        <v>46</v>
       </c>
       <c r="D2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3">
-        <v>1002</v>
-      </c>
-      <c r="B3" t="s">
-        <v>61</v>
-      </c>
-      <c r="C3">
-        <v>150</v>
-      </c>
-      <c r="D3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4">
-        <v>1003</v>
-      </c>
       <c r="B4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C4">
-        <v>120</v>
+        <v>45</v>
+      </c>
+      <c r="C4" t="s">
+        <v>48</v>
       </c>
       <c r="D4" t="s">
-        <v>44</v>
+        <v>51</v>
+      </c>
+      <c r="E4" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -944,40 +960,40 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4" t="s">
-        <v>7</v>
-      </c>
       <c r="B4" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -986,49 +1002,49 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C2">
         <v>1001</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C3">
         <v>1002</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C4">
         <v>1003</v>
@@ -1040,52 +1056,52 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>11</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B4" t="s">
         <v>28</v>
       </c>
-      <c r="C2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" t="s">
-        <v>30</v>
-      </c>
       <c r="C4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
cambiamenti estetica, pulsanti e filtri
in corso...........................
</commit_message>
<xml_diff>
--- a/Database_SpiaggiaFacile_Aggiornato.xlsx
+++ b/Database_SpiaggiaFacile_Aggiornato.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nocer\Documents\UNIVERSITA\1 Triennale UniBG\3 ANNO\9 PROGRAMMAZIONE WEB\PROGETTI\PRIMO\ProgettoWeb-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E27A5F3-579C-46FB-B4DC-09FD6DC49F20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A29104C1-7FD8-4128-A470-6FAF13FA466F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10660" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10660" firstSheet="3" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ombrelloni" sheetId="1" r:id="rId1"/>
     <sheet name="Tipologie" sheetId="2" r:id="rId2"/>
-    <sheet name="Contratti" sheetId="5" r:id="rId3"/>
+    <sheet name="Contratti" sheetId="9" r:id="rId3"/>
     <sheet name="Tariffa" sheetId="3" r:id="rId4"/>
     <sheet name="Cliente" sheetId="4" r:id="rId5"/>
     <sheet name="GiornoDisponibilita" sheetId="6" r:id="rId6"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="72">
   <si>
     <t>id</t>
   </si>
@@ -83,15 +83,6 @@
     <t>Luxury</t>
   </si>
   <si>
-    <t>Ombrellone base</t>
-  </si>
-  <si>
-    <t>Ampio con tavolino</t>
-  </si>
-  <si>
-    <t>Con lettini e cassaforte</t>
-  </si>
-  <si>
     <t>prezzo</t>
   </si>
   <si>
@@ -234,6 +225,24 @@
   </si>
   <si>
     <t>PostoFila</t>
+  </si>
+  <si>
+    <t>Ombrellone base, un lettino e una sdraio</t>
+  </si>
+  <si>
+    <t>Ombrellone con un lettino, due sdraio e tavolino</t>
+  </si>
+  <si>
+    <t>Ombrellone doppio, due lettini, tavolino e cassetta di sicurezza</t>
+  </si>
+  <si>
+    <t>lunedi,martedi</t>
+  </si>
+  <si>
+    <t>giovedi,sabato</t>
+  </si>
+  <si>
+    <t>venerdi,mercoledi</t>
   </si>
 </sst>
 </file>
@@ -612,10 +621,10 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>2</v>
@@ -681,6 +690,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="3" max="3" width="30.08984375" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
@@ -701,7 +713,7 @@
         <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -712,7 +724,7 @@
         <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>19</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
@@ -723,7 +735,7 @@
         <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>20</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>
@@ -732,22 +744,26 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C4F1886-A5AE-44BF-876F-2CABD6A556AA}">
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="11.90625" customWidth="1"/>
+    <col min="4" max="4" width="14.7265625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
@@ -755,13 +771,13 @@
         <v>1001</v>
       </c>
       <c r="B2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C2">
         <v>100</v>
       </c>
       <c r="D2" t="s">
-        <v>40</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -769,13 +785,13 @@
         <v>1002</v>
       </c>
       <c r="B3" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C3">
         <v>150</v>
       </c>
       <c r="D3" t="s">
-        <v>41</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -783,13 +799,13 @@
         <v>1003</v>
       </c>
       <c r="B4" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C4">
         <v>120</v>
       </c>
       <c r="D4" t="s">
-        <v>42</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -807,70 +823,70 @@
         <v>12</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B2">
         <v>20</v>
       </c>
       <c r="C2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" t="s">
         <v>29</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>32</v>
-      </c>
-      <c r="E2" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B3">
         <v>30</v>
       </c>
       <c r="C3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" t="s">
         <v>30</v>
       </c>
-      <c r="D3" t="s">
-        <v>33</v>
-      </c>
       <c r="E3" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B4">
         <v>40</v>
       </c>
       <c r="C4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" t="s">
         <v>31</v>
       </c>
-      <c r="D4" t="s">
-        <v>34</v>
-      </c>
       <c r="E4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="F4">
         <v>7</v>
@@ -894,64 +910,64 @@
         <v>13</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" t="s">
         <v>40</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>43</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>46</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>49</v>
-      </c>
-      <c r="E2" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" t="s">
         <v>41</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>44</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>47</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>50</v>
-      </c>
-      <c r="E3" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B4" t="s">
         <v>42</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>45</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>48</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>51</v>
-      </c>
-      <c r="E4" t="s">
-        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -966,10 +982,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
@@ -977,7 +993,7 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
@@ -985,7 +1001,7 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -993,7 +1009,7 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -1008,13 +1024,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
@@ -1022,7 +1038,7 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C2">
         <v>1001</v>
@@ -1033,7 +1049,7 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C3">
         <v>1002</v>
@@ -1044,7 +1060,7 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C4">
         <v>1003</v>
@@ -1062,13 +1078,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
@@ -1076,10 +1092,10 @@
         <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -1087,10 +1103,10 @@
         <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C3" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
@@ -1098,10 +1114,10 @@
         <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>